<commit_message>
Add description column to signal_android_lists.xlsx (120 rows, 3 columns)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/signal_android_lists.xlsx
+++ b/signal_android_lists.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Lists" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lists'!$A$1:$B$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lists'!$A$1:$C$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,11 +450,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B121"/>
+  <dimension ref="A1:C121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="67" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +469,11 @@
           <t>interface</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -480,6 +486,11 @@
           <t>chats</t>
         </is>
       </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>show all chats with preview, time, and unread</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -492,6 +503,11 @@
           <t>chats</t>
         </is>
       </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>filter the conversation list by folder</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -504,6 +520,11 @@
           <t>chats</t>
         </is>
       </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>show chats, contacts, and messages matching search</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -516,6 +537,11 @@
           <t>chats</t>
         </is>
       </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>pick a person to start or find a chat</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -528,6 +554,11 @@
           <t>archive</t>
         </is>
       </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>show chats moved out of the main list</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -540,6 +571,11 @@
           <t>calls</t>
         </is>
       </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>show recent voice and video calls</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -552,6 +588,11 @@
           <t>calls</t>
         </is>
       </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>show only missed calls after the filter is on</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -564,6 +605,11 @@
           <t>stories</t>
         </is>
       </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>show my story and others’ stories to open</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -576,6 +622,11 @@
           <t>settings</t>
         </is>
       </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>navigate to account, app, and support screens</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -588,6 +639,11 @@
           <t>settings</t>
         </is>
       </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>jump to a settings item by name</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -600,6 +656,11 @@
           <t>profile</t>
         </is>
       </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>open profile details and related actions</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -612,6 +673,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>show the thread of sent and received messages</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -624,6 +690,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>pick recent photos or videos to send</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -636,6 +707,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>choose gallery, file, location, contact, or other attach types</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -648,6 +724,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>browse device media to attach</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -660,6 +741,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>insert an emoji into the composer</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -672,6 +758,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>switch emoji groups</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -684,6 +775,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>pick a sticker to send</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -696,6 +792,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>switch installed sticker packs</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -708,6 +809,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>pick a GIF to send</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -720,6 +826,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>switch GIF search categories</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -732,6 +843,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>insert an @mention of a group member</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -744,6 +860,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>complete emoji, mention, or other inline queries</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -756,6 +877,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>offer stickers that match typed text</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -768,6 +894,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>show who reacted to a message</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -780,6 +911,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>show who voted for each poll option</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -792,6 +928,11 @@
           <t>conversation</t>
         </is>
       </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>list contacts whose safety number changed before send</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -804,6 +945,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>change mute, disappearing messages, wallpaper, and chat options</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -816,6 +962,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>show members and open a member</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -828,6 +979,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>browse photos, videos, and files in the chat</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -840,6 +996,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>show groups you share with this person</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -852,6 +1013,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>show invited people who have not joined</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -864,6 +1030,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>approve or deny join requests</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -876,6 +1047,11 @@
           <t>conversation settings</t>
         </is>
       </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>set custom notification sound and behavior</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -888,6 +1064,11 @@
           <t>account</t>
         </is>
       </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>manage phone number, PIN, and delete account</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -900,6 +1081,11 @@
           <t>linked devices</t>
         </is>
       </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>show and unlink paired desktops and devices</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -912,6 +1098,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>change theme, language, and icon</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -924,6 +1115,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>pick light, dark, or system theme</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -936,6 +1132,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>pick the app language</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -948,6 +1149,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>pick a bubble color</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -960,6 +1166,11 @@
           <t>appearance</t>
         </is>
       </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>pick a chat background</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -972,6 +1183,11 @@
           <t>chats settings</t>
         </is>
       </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>change keyboard, SMS, folders, and chat defaults</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -984,6 +1200,11 @@
           <t>chat folders</t>
         </is>
       </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>create and reorder chat folders</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -996,6 +1217,11 @@
           <t>chat folders</t>
         </is>
       </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>choose which chats belong in a folder</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1008,6 +1234,11 @@
           <t>stories privacy</t>
         </is>
       </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>choose who can see each story</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -1020,6 +1251,11 @@
           <t>stories privacy</t>
         </is>
       </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>add or remove people who can view a story</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1032,6 +1268,11 @@
           <t>notifications</t>
         </is>
       </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>turn message and call alerts on or off</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -1044,6 +1285,11 @@
           <t>notifications</t>
         </is>
       </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>pick or edit a notification profile</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1056,6 +1302,11 @@
           <t>notification profiles</t>
         </is>
       </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>choose who can notify you while a profile is on</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -1068,6 +1319,11 @@
           <t>privacy</t>
         </is>
       </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>open blocked list, screen lock, and disappearing defaults</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1080,6 +1336,11 @@
           <t>privacy</t>
         </is>
       </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>unblock or review blocked people</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -1092,6 +1353,11 @@
           <t>privacy</t>
         </is>
       </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>change relay calls and other advanced privacy options</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1104,6 +1370,11 @@
           <t>privacy</t>
         </is>
       </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>control who can see or find your number</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -1116,6 +1387,11 @@
           <t>privacy</t>
         </is>
       </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>pick a default disappearing-message timer</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1128,6 +1404,11 @@
           <t>backups settings</t>
         </is>
       </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>turn backups on and open backup details</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -1140,6 +1421,11 @@
           <t>remote backups</t>
         </is>
       </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>manage paid or cloud backup status and storage</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1152,6 +1438,11 @@
           <t>local backups</t>
         </is>
       </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>manage on-device backup files</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -1164,16 +1455,26 @@
           <t>backups type</t>
         </is>
       </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>choose a backup plan or type</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>data and storage settings list</t>
+          <t>data and storage list</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
           <t>data and storage</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>manage media quality, storage, and proxy</t>
         </is>
       </c>
     </row>
@@ -1188,6 +1489,11 @@
           <t>help</t>
         </is>
       </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>open support, debug log, licenses, and legal links</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1200,6 +1506,11 @@
           <t>help</t>
         </is>
       </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>show third-party licenses</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -1212,6 +1523,11 @@
           <t>labs</t>
         </is>
       </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>toggle experimental features</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1224,6 +1540,11 @@
           <t>internal</t>
         </is>
       </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>open debug and internal tools</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -1236,6 +1557,11 @@
           <t>internal</t>
         </is>
       </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>run internal search experiments</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1248,6 +1574,11 @@
           <t>internal</t>
         </is>
       </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>list internal issue shortcuts</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -1260,6 +1591,11 @@
           <t>internal</t>
         </is>
       </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>debug a single conversation</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1272,6 +1608,11 @@
           <t>internal sqlite</t>
         </is>
       </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>show query results from the internal playground</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -1284,6 +1625,11 @@
           <t>internal storage</t>
         </is>
       </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>inspect storage-service records</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1296,6 +1642,11 @@
           <t>app updates</t>
         </is>
       </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>control in-app update checks</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -1308,6 +1659,11 @@
           <t>linked device account</t>
         </is>
       </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>manage this device when it is not primary</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1320,6 +1676,11 @@
           <t>export account data</t>
         </is>
       </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>choose what account data to export</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -1332,6 +1693,11 @@
           <t>country picker</t>
         </is>
       </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>pick a country calling code</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1344,6 +1710,11 @@
           <t>restore method</t>
         </is>
       </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>choose Signal backup, local file, transfer, or skip</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -1356,6 +1727,11 @@
           <t>local backup</t>
         </is>
       </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>pick a backup file on the device</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1368,6 +1744,11 @@
           <t>story archive</t>
         </is>
       </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>reopen archived stories</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -1380,6 +1761,11 @@
           <t>story viewer</t>
         </is>
       </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>show who viewed a story</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1392,6 +1778,11 @@
           <t>story viewer</t>
         </is>
       </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>show replies to a story</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -1404,6 +1795,11 @@
           <t>story viewer</t>
         </is>
       </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>page through stories in a viewer</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1416,6 +1812,11 @@
           <t>media gallery</t>
         </is>
       </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>browse and multi-select media to send</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -1428,6 +1829,11 @@
           <t>media preview</t>
         </is>
       </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>jump between items in a preview</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1440,6 +1846,11 @@
           <t>media overview</t>
         </is>
       </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>browse all media in a chat by type</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -1452,6 +1863,11 @@
           <t>media send</t>
         </is>
       </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>review selected items before send</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1464,6 +1880,11 @@
           <t>sticker pack</t>
         </is>
       </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>preview stickers in a pack</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -1476,6 +1897,11 @@
           <t>sticker management</t>
         </is>
       </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>install, remove, or reorder sticker packs</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1488,6 +1914,11 @@
           <t>new chat</t>
         </is>
       </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>pick people to message</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -1500,6 +1931,11 @@
           <t>new group</t>
         </is>
       </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>pick members for a new group</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1512,6 +1948,11 @@
           <t>add members</t>
         </is>
       </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>add people to an existing group</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -1524,6 +1965,11 @@
           <t>share</t>
         </is>
       </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>pick chats to share incoming content into</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1536,6 +1982,11 @@
           <t>share</t>
         </is>
       </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>confirm recipients before send</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -1548,6 +1999,11 @@
           <t>find by</t>
         </is>
       </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>find someone by phone number or username</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1560,6 +2016,11 @@
           <t>call links</t>
         </is>
       </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>show call-link settings and members</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -1572,6 +2033,11 @@
           <t>call links</t>
         </is>
       </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>approve people waiting to join</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -1584,6 +2050,11 @@
           <t>in call</t>
         </is>
       </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>show extra participants who do not fit the grid</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -1596,6 +2067,11 @@
           <t>in call</t>
         </is>
       </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>pick a reaction during a call</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1608,6 +2084,11 @@
           <t>in call</t>
         </is>
       </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>switch speaker, earpiece, or headset</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -1620,6 +2101,11 @@
           <t>in call</t>
         </is>
       </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>admit or deny waiting callers</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -1632,6 +2118,11 @@
           <t>call quality</t>
         </is>
       </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>pick a call-quality problem to report</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -1644,6 +2135,11 @@
           <t>payments</t>
         </is>
       </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>show balance actions and recent payments</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -1656,6 +2152,11 @@
           <t>payments</t>
         </is>
       </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>show all payment transactions</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -1668,6 +2169,11 @@
           <t>payments</t>
         </is>
       </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>review payment details before send</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -1680,6 +2186,11 @@
           <t>payments recovery</t>
         </is>
       </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>show or confirm recovery-phrase words</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -1692,6 +2203,11 @@
           <t>donate</t>
         </is>
       </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>show past donation receipts</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -1704,6 +2220,11 @@
           <t>donate</t>
         </is>
       </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>enter bank-transfer details</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -1716,6 +2237,11 @@
           <t>donate</t>
         </is>
       </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>pick an iDEAL bank</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -1728,6 +2254,11 @@
           <t>username link</t>
         </is>
       </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>manage QR, color, and sharing</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -1740,6 +2271,11 @@
           <t>safety number</t>
         </is>
       </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>review connections after a safety-number change</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -1752,6 +2288,11 @@
           <t>review contacts</t>
         </is>
       </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>review possible contact or profile collisions</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -1764,6 +2305,11 @@
           <t>message details</t>
         </is>
       </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>show delivery and read status per person</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -1776,6 +2322,11 @@
           <t>contact share</t>
         </is>
       </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>pick which contact fields to send</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -1788,6 +2339,11 @@
           <t>contact share</t>
         </is>
       </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>edit a shared contact before send</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -1800,6 +2356,11 @@
           <t>nickname</t>
         </is>
       </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>edit nickname and note fields</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -1812,6 +2373,11 @@
           <t>create poll</t>
         </is>
       </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>add and reorder poll choices</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -1824,6 +2390,11 @@
           <t>wallpaper</t>
         </is>
       </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>preview wallpapers before apply</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -1836,6 +2407,11 @@
           <t>chat folders</t>
         </is>
       </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>pick a folder to put a chat in</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -1848,6 +2424,11 @@
           <t>username</t>
         </is>
       </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>explain username and QR options</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -1860,6 +2441,11 @@
           <t>payments</t>
         </is>
       </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>show MobileCoin ledger or debug lines</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -1872,6 +2458,11 @@
           <t>settings screens</t>
         </is>
       </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>render a generic settings screen as rows</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -1884,6 +2475,11 @@
           <t>settings screens</t>
         </is>
       </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>render older XML settings rows</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -1896,6 +2492,11 @@
           <t>contact search</t>
         </is>
       </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>search Signal and system contacts</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -1908,9 +2509,14 @@
           <t>chats search</t>
         </is>
       </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>bind typed search hits in the chats tab</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B121"/>
+  <autoFilter ref="A1:C121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>